<commit_message>
Use real CDX tenant users directly; remove profile mapping
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: 91e57aab-4107-4707-97d7-02508420b523
</commit_message>
<xml_diff>
--- a/agent-builder-copilot/Fargo_Dock_Schedule.xlsx
+++ b/agent-builder-copilot/Fargo_Dock_Schedule.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Megan Bowen</t>
+          <t>Lisa Taylor</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Megan Bowen</t>
+          <t>Lisa Taylor</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Anne Weiler</t>
+          <t>Sonia Rees</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Megan Bowen</t>
+          <t>Lisa Taylor</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Megan Bowen</t>
+          <t>Lisa Taylor</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Megan Bowen</t>
+          <t>Lisa Taylor</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Megan Bowen</t>
+          <t>Lisa Taylor</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Anne Weiler</t>
+          <t>Sonia Rees</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Recast to CDX users with a mailbox; guard against look-alike mailboxes; desktop log for every run
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: 91e57aab-4107-4707-97d7-02508420b523
</commit_message>
<xml_diff>
--- a/agent-builder-copilot/Fargo_Dock_Schedule.xlsx
+++ b/agent-builder-copilot/Fargo_Dock_Schedule.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Lisa Taylor</t>
+          <t>Teresa Sac</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Lisa Taylor</t>
+          <t>Teresa Sac</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Lisa Taylor</t>
+          <t>Teresa Sac</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Lisa Taylor</t>
+          <t>Teresa Sac</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Lisa Taylor</t>
+          <t>Teresa Sac</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Lisa Taylor</t>
+          <t>Teresa Sac</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">

</xml_diff>